<commit_message>
updated the may data and filter added
</commit_message>
<xml_diff>
--- a/Daywise_Distance_May_2026.xlsx
+++ b/Daywise_Distance_May_2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="40">
   <si>
     <t>Vehicle</t>
   </si>
@@ -118,34 +118,19 @@
     <t>31</t>
   </si>
   <si>
+    <t>JC 400 MH 15 JM 1385 - SWEEPER MASHINE</t>
+  </si>
+  <si>
+    <t>General</t>
+  </si>
+  <si>
     <t>JC 400 MH 15 JM 1384 - SWEEPER MACHINE</t>
   </si>
   <si>
-    <t>ELGIN</t>
-  </si>
-  <si>
-    <t>EAGLE</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
     <t>JC 400 MH 15 JM 1382 - SWEEPER MACHINE</t>
   </si>
   <si>
-    <t>General</t>
-  </si>
-  <si>
     <t>JC 400 MH 15 JM 1383 - SWEEPER MACHINE</t>
-  </si>
-  <si>
-    <t>JC 400 MH 15 JM 1385 - SWEEPER MACHINE</t>
-  </si>
-  <si>
-    <t>AMW</t>
-  </si>
-  <si>
-    <t>1618 TP</t>
   </si>
 </sst>
 </file>
@@ -168,7 +153,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -178,11 +163,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE6E6E6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF0000FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -213,7 +193,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -222,9 +202,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -694,100 +671,100 @@
         <v>36</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D2" s="3">
+        <v>1044</v>
+      </c>
+      <c r="E2" s="3">
+        <v>33</v>
+      </c>
+      <c r="F2" s="3">
+        <v>33</v>
+      </c>
+      <c r="G2" s="3">
+        <v>0</v>
+      </c>
+      <c r="H2" s="3">
+        <v>35</v>
+      </c>
+      <c r="I2" s="3">
+        <v>47</v>
+      </c>
+      <c r="J2" s="3">
+        <v>0</v>
+      </c>
+      <c r="K2" s="3">
         <v>37</v>
       </c>
-      <c r="D2" s="3">
-        <v>745</v>
-      </c>
-      <c r="E2" s="3">
-        <v>35</v>
-      </c>
-      <c r="F2" s="3">
-        <v>61</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="H2" s="3">
+      <c r="L2" s="3">
+        <v>43</v>
+      </c>
+      <c r="M2" s="3">
+        <v>40</v>
+      </c>
+      <c r="N2" s="3">
+        <v>0</v>
+      </c>
+      <c r="O2" s="3">
+        <v>36</v>
+      </c>
+      <c r="P2" s="3">
+        <v>43</v>
+      </c>
+      <c r="Q2" s="3">
+        <v>49</v>
+      </c>
+      <c r="R2" s="3">
+        <v>40</v>
+      </c>
+      <c r="S2" s="3">
+        <v>37</v>
+      </c>
+      <c r="T2" s="3">
+        <v>36</v>
+      </c>
+      <c r="U2" s="3">
+        <v>0</v>
+      </c>
+      <c r="V2" s="3">
+        <v>40</v>
+      </c>
+      <c r="W2" s="3">
         <v>54</v>
       </c>
-      <c r="I2" s="3">
-        <v>79</v>
-      </c>
-      <c r="J2" s="3">
-        <v>52</v>
-      </c>
-      <c r="K2" s="3">
-        <v>58</v>
-      </c>
-      <c r="L2" s="3">
-        <v>68</v>
-      </c>
-      <c r="M2" s="3">
-        <v>75</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="O2" s="3">
-        <v>88</v>
-      </c>
-      <c r="P2" s="3">
-        <v>51</v>
-      </c>
-      <c r="Q2" s="3">
-        <v>67</v>
-      </c>
-      <c r="R2" s="3">
-        <v>57</v>
-      </c>
-      <c r="S2" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="T2" s="3">
-        <v>0</v>
-      </c>
-      <c r="U2" s="3">
-        <v>0</v>
-      </c>
-      <c r="V2" s="3">
-        <v>0</v>
-      </c>
-      <c r="W2" s="3">
-        <v>0</v>
-      </c>
       <c r="X2" s="3">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="Y2" s="3">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="Z2" s="3">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="AA2" s="3">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="AB2" s="3">
         <v>0</v>
       </c>
       <c r="AC2" s="3">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="AD2" s="3">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="AE2" s="3">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="AF2" s="3">
         <v>0</v>
       </c>
       <c r="AG2" s="3">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="AH2" s="3">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="AI2" s="3">
         <v>0</v>
@@ -795,106 +772,106 @@
     </row>
     <row r="3" ht="54" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" s="3">
+        <v>1142</v>
+      </c>
+      <c r="E3" s="3">
+        <v>41</v>
+      </c>
+      <c r="F3" s="3">
+        <v>48</v>
+      </c>
+      <c r="G3" s="3">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3">
+        <v>47</v>
+      </c>
+      <c r="I3" s="3">
         <v>40</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" s="3">
-        <v>600</v>
-      </c>
-      <c r="E3" s="3">
-        <v>67</v>
-      </c>
-      <c r="F3" s="3">
-        <v>56</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="H3" s="3">
-        <v>66</v>
-      </c>
-      <c r="I3" s="3">
-        <v>43</v>
-      </c>
       <c r="J3" s="3">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="K3" s="3">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="L3" s="3">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="M3" s="3">
-        <v>53</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
+      </c>
+      <c r="N3" s="3">
+        <v>0</v>
       </c>
       <c r="O3" s="3">
-        <v>65</v>
+        <v>44</v>
       </c>
       <c r="P3" s="3">
+        <v>46</v>
+      </c>
+      <c r="Q3" s="3">
+        <v>34</v>
+      </c>
+      <c r="R3" s="3">
+        <v>49</v>
+      </c>
+      <c r="S3" s="3">
+        <v>48</v>
+      </c>
+      <c r="T3" s="3">
+        <v>44</v>
+      </c>
+      <c r="U3" s="3">
+        <v>0</v>
+      </c>
+      <c r="V3" s="3">
+        <v>51</v>
+      </c>
+      <c r="W3" s="3">
+        <v>73</v>
+      </c>
+      <c r="X3" s="3">
+        <v>57</v>
+      </c>
+      <c r="Y3" s="3">
         <v>42</v>
       </c>
-      <c r="Q3" s="3">
-        <v>41</v>
-      </c>
-      <c r="R3" s="3">
+      <c r="Z3" s="3">
+        <v>45</v>
+      </c>
+      <c r="AA3" s="3">
         <v>42</v>
       </c>
-      <c r="S3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="T3" s="3">
-        <v>0</v>
-      </c>
-      <c r="U3" s="3">
-        <v>0</v>
-      </c>
-      <c r="V3" s="3">
-        <v>0</v>
-      </c>
-      <c r="W3" s="3">
-        <v>0</v>
-      </c>
-      <c r="X3" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y3" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z3" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="3">
-        <v>0</v>
-      </c>
       <c r="AB3" s="3">
         <v>0</v>
       </c>
       <c r="AC3" s="3">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="AD3" s="3">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="AE3" s="3">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="AF3" s="3">
         <v>0</v>
       </c>
       <c r="AG3" s="3">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="AH3" s="3">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="AI3" s="3">
         <v>0</v>
@@ -902,106 +879,106 @@
     </row>
     <row r="4" ht="54" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>36</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D4" s="3">
-        <v>547</v>
+        <v>1007</v>
       </c>
       <c r="E4" s="3">
+        <v>33</v>
+      </c>
+      <c r="F4" s="3">
+        <v>38</v>
+      </c>
+      <c r="G4" s="3">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3">
+        <v>33</v>
+      </c>
+      <c r="I4" s="3">
+        <v>42</v>
+      </c>
+      <c r="J4" s="3">
+        <v>44</v>
+      </c>
+      <c r="K4" s="3">
+        <v>40</v>
+      </c>
+      <c r="L4" s="3">
+        <v>39</v>
+      </c>
+      <c r="M4" s="3">
         <v>41</v>
       </c>
-      <c r="F4" s="3">
-        <v>54</v>
-      </c>
-      <c r="G4" s="3">
-        <v>0</v>
-      </c>
-      <c r="H4" s="3">
-        <v>44</v>
-      </c>
-      <c r="I4" s="3">
-        <v>43</v>
-      </c>
-      <c r="J4" s="3">
-        <v>63</v>
-      </c>
-      <c r="K4" s="3">
-        <v>36</v>
-      </c>
-      <c r="L4" s="3">
-        <v>51</v>
-      </c>
-      <c r="M4" s="3">
-        <v>45</v>
-      </c>
       <c r="N4" s="3">
         <v>0</v>
       </c>
       <c r="O4" s="3">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="P4" s="3">
         <v>42</v>
       </c>
       <c r="Q4" s="3">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="R4" s="3">
+        <v>42</v>
+      </c>
+      <c r="S4" s="3">
+        <v>35</v>
+      </c>
+      <c r="T4" s="3">
+        <v>35</v>
+      </c>
+      <c r="U4" s="3">
+        <v>0</v>
+      </c>
+      <c r="V4" s="3">
+        <v>0</v>
+      </c>
+      <c r="W4" s="3">
+        <v>66</v>
+      </c>
+      <c r="X4" s="3">
+        <v>60</v>
+      </c>
+      <c r="Y4" s="3">
+        <v>42</v>
+      </c>
+      <c r="Z4" s="3">
+        <v>43</v>
+      </c>
+      <c r="AA4" s="3">
+        <v>35</v>
+      </c>
+      <c r="AB4" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="3">
         <v>45</v>
       </c>
-      <c r="S4" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="T4" s="3">
-        <v>0</v>
-      </c>
-      <c r="U4" s="3">
-        <v>0</v>
-      </c>
-      <c r="V4" s="3">
-        <v>0</v>
-      </c>
-      <c r="W4" s="3">
-        <v>0</v>
-      </c>
-      <c r="X4" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z4" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA4" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB4" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC4" s="3">
-        <v>0</v>
-      </c>
       <c r="AD4" s="3">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="AE4" s="3">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="AF4" s="3">
         <v>0</v>
       </c>
       <c r="AG4" s="3">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="AH4" s="3">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="AI4" s="3">
         <v>0</v>
@@ -1009,106 +986,106 @@
     </row>
     <row r="5" ht="54" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="D5" s="3">
-        <v>474</v>
+        <v>1304</v>
       </c>
       <c r="E5" s="3">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="F5" s="3">
-        <v>41</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>38</v>
+        <v>50</v>
+      </c>
+      <c r="G5" s="3">
+        <v>0</v>
       </c>
       <c r="H5" s="3">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="I5" s="3">
-        <v>34</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>38</v>
+        <v>48</v>
+      </c>
+      <c r="J5" s="3">
+        <v>51</v>
       </c>
       <c r="K5" s="3">
         <v>47</v>
       </c>
       <c r="L5" s="3">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="M5" s="3">
         <v>50</v>
       </c>
-      <c r="N5" s="4" t="s">
-        <v>38</v>
+      <c r="N5" s="3">
+        <v>0</v>
       </c>
       <c r="O5" s="3">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="P5" s="3">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="Q5" s="3">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="R5" s="3">
-        <v>38</v>
-      </c>
-      <c r="S5" s="4" t="s">
-        <v>38</v>
+        <v>51</v>
+      </c>
+      <c r="S5" s="3">
+        <v>53</v>
       </c>
       <c r="T5" s="3">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="U5" s="3">
         <v>0</v>
       </c>
       <c r="V5" s="3">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="W5" s="3">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="X5" s="3">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="Y5" s="3">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="Z5" s="3">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="AA5" s="3">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="AB5" s="3">
         <v>0</v>
       </c>
       <c r="AC5" s="3">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="AD5" s="3">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="AE5" s="3">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="AF5" s="3">
         <v>0</v>
       </c>
       <c r="AG5" s="3">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="AH5" s="3">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="AI5" s="3">
         <v>0</v>
@@ -1116,6 +1093,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>